<commit_message>
Refactor ExcelToRevit command (v3) and UI
Refactor ExcelToRevitCommand to v3: make RunImportWorkflow static, add ExternalEvent/ReopenHandler to reopen the dialog, convert SyncStatusWindow to a non-persistent toast, and add a FileSystemWatcher with debounce to watch Excel files. Improve error handling, temp PNG cleanup, and import flow (create ImageType/ImageInstance and apply scale). Update SyncStatusWindow.xaml and its code-behind, and modify ExcelToRevitCommand.cs accordingly. Remove SKILL.md and ArcTool_Instructions.md. Also include updated VS workspace metadata, Copilot snapshots/indices and build/obj artifacts.
</commit_message>
<xml_diff>
--- a/ArcTool.TestConsole/Testconsole.xlsx
+++ b/ArcTool.TestConsole/Testconsole.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zcgp4-my.sharepoint.com/personal/duyquang868_zcgp4_onmicrosoft_com/Documents/Plugin Revit/ArcTool/ArcTool.TestConsole/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="109" documentId="13_ncr:1_{A605C092-534C-435B-BAEA-83AE92C65CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6846A24-2908-4281-B2C2-E7EBD1A6C1FB}"/>
+  <xr:revisionPtr revIDLastSave="291" documentId="13_ncr:1_{A605C092-534C-435B-BAEA-83AE92C65CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A10696A-00D5-47E2-9376-F95BE86079FB}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="0" windowWidth="27975" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="22">
   <si>
     <t>dsaf</t>
   </si>
@@ -55,6 +55,48 @@
   </si>
   <si>
     <t>adfasd</t>
+  </si>
+  <si>
+    <t>sfasf</t>
+  </si>
+  <si>
+    <t>eqfwf</t>
+  </si>
+  <si>
+    <t>asdfad</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>asfd213</t>
+  </si>
+  <si>
+    <t>asfdasdf</t>
+  </si>
+  <si>
+    <t>dsf</t>
+  </si>
+  <si>
+    <t>fasdf</t>
+  </si>
+  <si>
+    <t>asdfasf</t>
+  </si>
+  <si>
+    <t>sdfafd</t>
+  </si>
+  <si>
+    <t>asfasdf</t>
+  </si>
+  <si>
+    <t>sdfas</t>
+  </si>
+  <si>
+    <t>asdfas</t>
+  </si>
+  <si>
+    <t>sdfasdf</t>
   </si>
 </sst>
 </file>
@@ -1301,7 +1343,9 @@
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -1325,15 +1369,21 @@
       <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="1"/>
+      <c r="C4" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
+      <c r="F4" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="G4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
+      <c r="I4" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -1341,7 +1391,9 @@
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
+      <c r="E5" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -1350,12 +1402,16 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
+      <c r="B6" s="1" t="s">
+        <v>4</v>
+      </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
+      <c r="G6" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
@@ -1363,9 +1419,13 @@
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
+      <c r="C7" s="1" t="s">
+        <v>4</v>
+      </c>
       <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
+      <c r="E7" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
@@ -1375,9 +1435,13 @@
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
+      <c r="C8" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
+      <c r="E8" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
@@ -1391,21 +1455,31 @@
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
+      <c r="E9" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
+      <c r="I9" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
+      <c r="B10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
+      <c r="E10" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
@@ -1417,19 +1491,31 @@
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
+      <c r="E11" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
+      <c r="G11" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
+      <c r="J11" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+      <c r="B12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
+      <c r="E12" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -1443,7 +1529,9 @@
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
+      <c r="E13" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
         <v>5</v>

</xml_diff>